<commit_message>
feat: Implement MLP builder and related functionality; update project structure and documentation
</commit_message>
<xml_diff>
--- a/docs/gabarito.xlsx
+++ b/docs/gabarito.xlsx
@@ -1,27 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aluno\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DevProjects\mlp-app\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1F1AB0-8C02-4D5F-9E39-1F6DA54337B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7035"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
     <sheet name="Plan2" sheetId="2" r:id="rId2"/>
     <sheet name="Plan3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>netC</t>
   </si>
@@ -93,12 +94,33 @@
   </si>
   <si>
     <t>EGSimples</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Wcb</t>
+  </si>
+  <si>
+    <t>Wdb</t>
+  </si>
+  <si>
+    <t>Desejado (F)</t>
+  </si>
+  <si>
+    <t>Desejado (G)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -143,10 +165,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -165,9 +188,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Escritório">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -205,9 +228,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Escritório">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -242,7 +265,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -277,7 +300,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Escritório">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -450,248 +473,293 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I22"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>0</v>
       </c>
-      <c r="B2">
+      <c r="B5">
+        <f>A2*G5+B2*G7</f>
         <v>1.2</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F2">
+      <c r="F5">
         <v>1</v>
       </c>
-      <c r="G2">
+      <c r="G5">
         <v>1.2</v>
       </c>
-      <c r="I2">
-        <f>1.2+1*B4*F2</f>
+      <c r="I5">
+        <f>1.2+1*B7*F5</f>
         <v>-44.564481116985604</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>1</v>
       </c>
-      <c r="B3">
-        <f>(1.2^2)/5</f>
+      <c r="B6">
+        <f>(B5^2)/5</f>
         <v>0.28799999999999998</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F3">
+      <c r="F6">
         <v>1</v>
       </c>
-      <c r="G3">
+      <c r="G6">
         <v>3.5</v>
       </c>
-      <c r="I3">
-        <f>3.5+1*B9*1</f>
+      <c r="I6">
+        <f>3.5+1*B12*1</f>
         <v>-210.17506708115681</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <f>(B14*2+B19*1.5)*(2*B2/5)</f>
-        <v>-45.764481116985607</v>
-      </c>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <f>(B17*G15+B22*G18)*(2*B5/5)</f>
+        <v>-45.764481116985607</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>2</v>
       </c>
-      <c r="B7">
+      <c r="B10">
+        <f>A2*G6+B2*G8</f>
         <v>3.5</v>
       </c>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>3</v>
       </c>
-      <c r="B8">
-        <f>B7^2/5</f>
+      <c r="B11">
+        <f>B10^2/5</f>
         <v>2.4500000000000002</v>
       </c>
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9">
-        <f>(B14*3.2+B19*(-1.1))*(2*B7/5)</f>
-        <v>-213.67506708115681</v>
-      </c>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E11" s="2"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B12">
-        <f>B3*2+B8*3.2</f>
-        <v>8.4160000000000004</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12">
-        <v>0.28799999999999998</v>
-      </c>
-      <c r="G12">
-        <v>2</v>
-      </c>
-      <c r="I12">
-        <f>G12+1*B14*F12</f>
-        <v>-11.734082605219841</v>
-      </c>
+        <f>(B17*3.2+B22*(-1.1))*(2*B10/5)</f>
+        <v>-213.67506708115681</v>
+      </c>
+      <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13">
-        <f>B12^2/5</f>
-        <v>14.165811200000002</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F13">
-        <v>2.4500000000000002</v>
-      </c>
-      <c r="G13">
-        <v>3.2</v>
-      </c>
-      <c r="I13">
-        <f>G13+1*B14*F13</f>
-        <v>-113.63507771801602</v>
-      </c>
+      <c r="E13" s="2"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>8</v>
-      </c>
-      <c r="B14">
-        <f>(0-B13)*(2*B12/5)</f>
-        <v>-47.687786823680007</v>
-      </c>
       <c r="E14" s="2"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="B15">
-        <f>(0-B13)</f>
-        <v>-14.165811200000002</v>
+        <f>B6*G15+B11*G16</f>
+        <v>8.4160000000000004</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F15">
         <v>0.28799999999999998</v>
       </c>
       <c r="G15">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="I15">
-        <f>G15+1*B19*F15</f>
-        <v>1.50631769349888</v>
+        <f>G15+1*B17*F15</f>
+        <v>-11.734082605219841</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16">
+        <f>B15^2/5</f>
+        <v>14.165811200000002</v>
+      </c>
       <c r="E16" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F16">
         <v>2.4500000000000002</v>
       </c>
       <c r="G16">
+        <v>3.2</v>
+      </c>
+      <c r="I16">
+        <f>G16+1*B17*F16</f>
+        <v>-113.63507771801602</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17">
+        <f>(D2-B16)*(2*B15/5)</f>
+        <v>-47.687786823680007</v>
+      </c>
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18">
+        <f>(D2-B16)</f>
+        <v>-14.165811200000002</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18">
+        <v>0.28799999999999998</v>
+      </c>
+      <c r="G18">
+        <v>1.5</v>
+      </c>
+      <c r="I18">
+        <f>G18+1*B22*F18</f>
+        <v>1.50631769349888</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19">
+        <v>2.4500000000000002</v>
+      </c>
+      <c r="G19">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="I16">
-        <f>G16+1*B19*F16</f>
+      <c r="I19">
+        <f>G19+1*B22*F19</f>
         <v>-1.0462557323879991</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>6</v>
       </c>
-      <c r="B17">
-        <f>B3*1.5+B8*(-1.1)</f>
+      <c r="B20">
+        <f>B6*G18+B11*G19</f>
         <v>-2.2630000000000003</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>7</v>
       </c>
-      <c r="B18">
-        <f>B17^2/5</f>
+      <c r="B21">
+        <f>B20^2/5</f>
         <v>1.0242338000000004</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>9</v>
       </c>
-      <c r="B19">
-        <f>(1-B18)*(2*B17/5)</f>
+      <c r="B22">
+        <f>(E2-B21)*(2*B20/5)</f>
         <v>2.1936435760000379E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>23</v>
       </c>
-      <c r="B20">
-        <f>(1-B18)</f>
+      <c r="B23">
+        <f>(E2-B21)</f>
         <v>-2.4233800000000416E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>12</v>
       </c>
-      <c r="B22">
-        <f>0.5*(B20^2+B15^2)</f>
+      <c r="B25">
+        <f>0.5*(B23^2+B18^2)</f>
         <v>100.33539711555397</v>
       </c>
     </row>
@@ -702,7 +770,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -711,7 +779,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>